<commit_message>
Mejoras para exportacion de aplicacion
</commit_message>
<xml_diff>
--- a/Syllabus_Electronica/Ingeniería en Control y Automatización/Área Profesional/Electivas/24711 - Telecomunicaciones Aeronáuticas.xlsx
+++ b/Syllabus_Electronica/Ingeniería en Control y Automatización/Área Profesional/Electivas/24711 - Telecomunicaciones Aeronáuticas.xlsx
@@ -892,7 +892,7 @@
       <c r="F3" s="34" t="inlineStr">
         <is>
           <t>Fecha de Aprobación:
-22/02/2025</t>
+01/01/2000</t>
         </is>
       </c>
       <c r="G3" s="45" t="n"/>
@@ -1633,9 +1633,9 @@
     <mergeCell ref="A12:I12"/>
     <mergeCell ref="H40:I40"/>
     <mergeCell ref="A6:B6"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="A1:B3"/>
     <mergeCell ref="A26:I26"/>
-    <mergeCell ref="A1:B3"/>
-    <mergeCell ref="H9:I9"/>
     <mergeCell ref="C2:E2"/>
     <mergeCell ref="A21:I21"/>
     <mergeCell ref="A33:I33"/>

</xml_diff>